<commit_message>
chore(data-release): publish site data 2026-09-11 06:09:47 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -18409,13 +18409,13 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>42567</v>
+        <v>41466</v>
       </c>
       <c r="O115" t="n">
-        <v>42567</v>
+        <v>41466</v>
       </c>
       <c r="R115" t="n">
-        <v>19.93185452196065</v>
+        <v>19.41631497656918</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -18989,13 +18989,13 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1258</v>
+        <v>1422</v>
       </c>
       <c r="O119" t="n">
-        <v>1258</v>
+        <v>1422</v>
       </c>
       <c r="R119" t="n">
-        <v>0.5890542671230413</v>
+        <v>0.665846715301244</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -19134,13 +19134,13 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>11345</v>
+        <v>11649</v>
       </c>
       <c r="O120" t="n">
-        <v>11345</v>
+        <v>11649</v>
       </c>
       <c r="R120" t="n">
-        <v>5.31225807671773</v>
+        <v>5.454605053828544</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -20397,13 +20397,13 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>37468</v>
+        <v>39979</v>
       </c>
       <c r="O128" t="n">
-        <v>37468</v>
+        <v>39979</v>
       </c>
       <c r="R128" t="n">
-        <v>17.54426492890788</v>
+        <v>18.7200322299778</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
@@ -20687,13 +20687,13 @@
         </is>
       </c>
       <c r="N130" t="n">
-        <v>244</v>
+        <v>416</v>
       </c>
       <c r="O130" t="n">
-        <v>244</v>
+        <v>416</v>
       </c>
       <c r="R130" t="n">
-        <v>0.1142521789968379</v>
+        <v>0.194790600256904</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -20832,13 +20832,13 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>6520</v>
+        <v>7678</v>
       </c>
       <c r="O131" t="n">
-        <v>6520</v>
+        <v>7678</v>
       </c>
       <c r="R131" t="n">
-        <v>3.052968061718784</v>
+        <v>3.595197665318531</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -21733,6 +21733,296 @@
         </is>
       </c>
       <c r="BC136" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>D021</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Dengue</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>登革热</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N137" t="n">
+        <v>4484</v>
+      </c>
+      <c r="O137" t="n">
+        <v>4484</v>
+      </c>
+      <c r="R137" t="n">
+        <v>2.099617912384513</v>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO137" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP137" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR137" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS137" t="inlineStr"/>
+      <c r="AT137" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU137" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV137" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW137" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX137" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY137" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ137" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA137" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB137" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC137" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>D052</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Chikungunya</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>基孔肯雅热</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N138" t="n">
+        <v>451</v>
+      </c>
+      <c r="O138" t="n">
+        <v>451</v>
+      </c>
+      <c r="R138" t="n">
+        <v>0.211179232490057</v>
+      </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO138" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP138" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR138" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS138" t="inlineStr"/>
+      <c r="AT138" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU138" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV138" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW138" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX138" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY138" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ138" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA138" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB138" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC138" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -21771,7 +22061,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
@@ -21854,7 +22144,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
@@ -21864,7 +22154,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11">
@@ -21916,7 +22206,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1101790</v>
+        <v>1109933</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-13 13:21:47 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -19975,17 +19975,17 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -20004,13 +20004,13 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>1597</v>
+        <v>1253</v>
       </c>
       <c r="O126" t="n">
-        <v>1597</v>
+        <v>1253</v>
       </c>
       <c r="R126" t="n">
-        <v>0.7477898764670088</v>
+        <v>0.5867130339468767</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
@@ -20019,7 +20019,7 @@
       </c>
       <c r="U126" t="inlineStr">
         <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AA126" t="inlineStr">
@@ -20029,7 +20029,7 @@
       </c>
       <c r="AO126" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP126" t="inlineStr">
@@ -20039,12 +20039,12 @@
       </c>
       <c r="AQ126" t="inlineStr">
         <is>
-          <t>legacy_gap_fill</t>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS126" t="inlineStr">
         <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT126" t="n">
@@ -20052,7 +20052,7 @@
       </c>
       <c r="AU126" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV126" t="inlineStr">
@@ -20134,17 +20134,17 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -20163,19 +20163,19 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>1597</v>
+        <v>1253</v>
       </c>
       <c r="O127" t="n">
-        <v>1597</v>
+        <v>1253</v>
       </c>
       <c r="U127" t="inlineStr">
         <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="V127" t="inlineStr">
         <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="W127" t="inlineStr">
@@ -20185,7 +20185,7 @@
       </c>
       <c r="X127" t="inlineStr">
         <is>
-          <t>Meningitis</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr">
@@ -20225,12 +20225,12 @@
       </c>
       <c r="AF127" t="inlineStr">
         <is>
-          <t>conditional</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="AG127" t="inlineStr">
         <is>
-          <t>reported_aggregate</t>
+          <t>non_additive</t>
         </is>
       </c>
       <c r="AH127" t="inlineStr">
@@ -20245,17 +20245,17 @@
       </c>
       <c r="AJ127" t="inlineStr">
         <is>
-          <t>BR_SINAN_MENI_current</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK127" t="inlineStr">
         <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
         </is>
       </c>
       <c r="AM127" t="inlineStr">
         <is>
-          <t>provisional</t>
+          <t>final; provisional</t>
         </is>
       </c>
       <c r="AN127" t="b">
@@ -20263,7 +20263,7 @@
       </c>
       <c r="AO127" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP127" t="inlineStr">
@@ -20273,12 +20273,12 @@
       </c>
       <c r="AQ127" t="inlineStr">
         <is>
-          <t>legacy_gap_fill</t>
+          <t>parity</t>
         </is>
       </c>
       <c r="AS127" t="inlineStr">
         <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT127" t="n">
@@ -20286,7 +20286,7 @@
       </c>
       <c r="AU127" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV127" t="inlineStr">
@@ -20368,70 +20368,84 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N128" t="n">
-        <v>39979</v>
+        <v>548</v>
       </c>
       <c r="O128" t="n">
-        <v>39979</v>
+        <v>548</v>
       </c>
       <c r="R128" t="n">
-        <v>18.7200322299778</v>
+        <v>0.2565991561076524</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO128" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP128" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR128" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS128" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ128" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS128" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT128" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU128" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV128" t="inlineStr">
@@ -20498,7 +20512,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -20513,70 +20527,159 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N129" t="n">
-        <v>41</v>
+        <v>548</v>
       </c>
       <c r="O129" t="n">
-        <v>41</v>
-      </c>
-      <c r="R129" t="n">
-        <v>0.01919811204455063</v>
-      </c>
-      <c r="S129" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>548</v>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>SINAN MENT work-related mental disorder notifications.</t>
+        </is>
+      </c>
+      <c r="AM129" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN129" t="b">
+        <v>1</v>
       </c>
       <c r="AO129" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP129" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR129" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS129" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ129" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS129" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU129" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV129" t="inlineStr">
@@ -20658,42 +20761,42 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D194</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Noise-induced hearing loss</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>噪声性听力损失</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N130" t="n">
-        <v>416</v>
+        <v>60</v>
       </c>
       <c r="O130" t="n">
-        <v>416</v>
+        <v>60</v>
       </c>
       <c r="R130" t="n">
-        <v>0.194790600256904</v>
+        <v>0.02809479811397654</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -20803,42 +20906,42 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D195</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Pneumoconiosis</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>尘肺病</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N131" t="n">
-        <v>7678</v>
+        <v>22</v>
       </c>
       <c r="O131" t="n">
-        <v>7678</v>
+        <v>22</v>
       </c>
       <c r="R131" t="n">
-        <v>3.595197665318531</v>
+        <v>0.01030142597512473</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -20948,70 +21051,84 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N132" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="O132" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="R132" t="n">
-        <v>0.004214219717096481</v>
+        <v>0.7477898764670088</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO132" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP132" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR132" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS132" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ132" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS132" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT132" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU132" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV132" t="inlineStr">
@@ -21078,7 +21195,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -21093,17 +21210,17 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -21113,50 +21230,139 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N133" t="n">
+        <v>1597</v>
+      </c>
+      <c r="O133" t="n">
+        <v>1597</v>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W133" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X133" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y133" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z133" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA133" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC133" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD133" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE133" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF133" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG133" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH133" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI133" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ133" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK133" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM133" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN133" t="b">
         <v>1</v>
       </c>
-      <c r="O133" t="n">
+      <c r="AO133" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP133" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ133" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS133" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT133" t="n">
         <v>1</v>
       </c>
-      <c r="R133" t="n">
-        <v>0.0004682466352329422</v>
-      </c>
-      <c r="S133" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
-      <c r="AO133" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AP133" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR133" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS133" t="inlineStr"/>
-      <c r="AT133" t="n">
-        <v>0</v>
-      </c>
       <c r="AU133" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV133" t="inlineStr">
@@ -21238,22 +21444,22 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L134" t="inlineStr">
@@ -21267,13 +21473,13 @@
         </is>
       </c>
       <c r="N134" t="n">
-        <v>2970</v>
+        <v>39979</v>
       </c>
       <c r="O134" t="n">
-        <v>2970</v>
+        <v>39979</v>
       </c>
       <c r="R134" t="n">
-        <v>1.390692506641839</v>
+        <v>18.7200322299778</v>
       </c>
       <c r="S134" t="inlineStr">
         <is>
@@ -21383,22 +21589,22 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L135" t="inlineStr">
@@ -21412,55 +21618,41 @@
         </is>
       </c>
       <c r="N135" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="O135" t="n">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="R135" t="n">
-        <v>0.004682466352329423</v>
+        <v>0.01919811204455063</v>
       </c>
       <c r="S135" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA135" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO135" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP135" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ135" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS135" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR135" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS135" t="inlineStr"/>
       <c r="AT135" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU135" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV135" t="inlineStr">
@@ -21527,7 +21719,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -21542,22 +21734,22 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -21571,130 +21763,41 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>10</v>
+        <v>416</v>
       </c>
       <c r="O136" t="n">
-        <v>10</v>
-      </c>
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="V136" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W136" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X136" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y136" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z136" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="AA136" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB136" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC136" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD136" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE136" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF136" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG136" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH136" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI136" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ136" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK136" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM136" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN136" t="b">
-        <v>1</v>
+        <v>416</v>
+      </c>
+      <c r="R136" t="n">
+        <v>0.194790600256904</v>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="AO136" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP136" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ136" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS136" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR136" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS136" t="inlineStr"/>
       <c r="AT136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU136" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV136" t="inlineStr">
@@ -21776,17 +21879,17 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -21796,22 +21899,22 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N137" t="n">
-        <v>4484</v>
+        <v>7678</v>
       </c>
       <c r="O137" t="n">
-        <v>4484</v>
+        <v>7678</v>
       </c>
       <c r="R137" t="n">
-        <v>2.099617912384513</v>
+        <v>3.595197665318531</v>
       </c>
       <c r="S137" t="inlineStr">
         <is>
@@ -21921,42 +22024,42 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>451</v>
+        <v>9</v>
       </c>
       <c r="O138" t="n">
-        <v>451</v>
+        <v>9</v>
       </c>
       <c r="R138" t="n">
-        <v>0.211179232490057</v>
+        <v>0.004214219717096481</v>
       </c>
       <c r="S138" t="inlineStr">
         <is>
@@ -22023,6 +22126,2055 @@
         </is>
       </c>
       <c r="BC138" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>D178</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Acute flaccid paralysis</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>急性无力肢体麻痹</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N139" t="n">
+        <v>1</v>
+      </c>
+      <c r="O139" t="n">
+        <v>1</v>
+      </c>
+      <c r="R139" t="n">
+        <v>0.0004682466352329422</v>
+      </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO139" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP139" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR139" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS139" t="inlineStr"/>
+      <c r="AT139" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU139" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV139" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW139" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX139" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY139" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ139" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA139" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB139" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC139" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>D184</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Accident caused by venomous animals</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>毒性动物伤害</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N140" t="n">
+        <v>2970</v>
+      </c>
+      <c r="O140" t="n">
+        <v>2970</v>
+      </c>
+      <c r="R140" t="n">
+        <v>1.390692506641839</v>
+      </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO140" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP140" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR140" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS140" t="inlineStr"/>
+      <c r="AT140" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU140" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV140" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW140" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX140" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY140" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ140" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA140" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB140" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC140" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>D192</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Work-related repetitive strain injury</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>职业相关重复性劳损</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N141" t="n">
+        <v>391</v>
+      </c>
+      <c r="O141" t="n">
+        <v>391</v>
+      </c>
+      <c r="R141" t="n">
+        <v>0.1830844343760804</v>
+      </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="AA141" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO141" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP141" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ141" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS141" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="AT141" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU141" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV141" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW141" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX141" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY141" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ141" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA141" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB141" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC141" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>D192</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Work-related repetitive strain injury</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>职业相关重复性劳损</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N142" t="n">
+        <v>391</v>
+      </c>
+      <c r="O142" t="n">
+        <v>391</v>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="W142" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X142" t="inlineStr">
+        <is>
+          <t>Work-related repetitive strain injury</t>
+        </is>
+      </c>
+      <c r="Y142" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z142" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA142" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB142" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC142" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD142" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE142" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF142" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG142" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH142" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI142" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ142" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
+        </is>
+      </c>
+      <c r="AK142" t="inlineStr">
+        <is>
+          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
+        </is>
+      </c>
+      <c r="AM142" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN142" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO142" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP142" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ142" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS142" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="AT142" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU142" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV142" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW142" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX142" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY142" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ142" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA142" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB142" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC142" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>D193</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>职业相关精神障碍</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N143" t="n">
+        <v>172</v>
+      </c>
+      <c r="O143" t="n">
+        <v>172</v>
+      </c>
+      <c r="R143" t="n">
+        <v>0.08053842126006606</v>
+      </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="AA143" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO143" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP143" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ143" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS143" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="AT143" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU143" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV143" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW143" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX143" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY143" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ143" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA143" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB143" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC143" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>D193</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>职业相关精神障碍</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N144" t="n">
+        <v>172</v>
+      </c>
+      <c r="O144" t="n">
+        <v>172</v>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="W144" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X144" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="Y144" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z144" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA144" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB144" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC144" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD144" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE144" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF144" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG144" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH144" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI144" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ144" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
+        </is>
+      </c>
+      <c r="AK144" t="inlineStr">
+        <is>
+          <t>SINAN MENT work-related mental disorder notifications.</t>
+        </is>
+      </c>
+      <c r="AM144" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN144" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO144" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP144" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ144" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS144" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="AT144" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU144" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV144" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW144" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX144" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY144" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ144" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA144" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB144" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC144" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>D194</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Noise-induced hearing loss</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>噪声性听力损失</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N145" t="n">
+        <v>14</v>
+      </c>
+      <c r="O145" t="n">
+        <v>14</v>
+      </c>
+      <c r="R145" t="n">
+        <v>0.006555452893261191</v>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO145" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP145" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR145" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS145" t="inlineStr"/>
+      <c r="AT145" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU145" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV145" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW145" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX145" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY145" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ145" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA145" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB145" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC145" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>D195</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Pneumoconiosis</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>尘肺病</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N146" t="n">
+        <v>7</v>
+      </c>
+      <c r="O146" t="n">
+        <v>7</v>
+      </c>
+      <c r="R146" t="n">
+        <v>0.003277726446630596</v>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO146" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP146" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR146" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS146" t="inlineStr"/>
+      <c r="AT146" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU146" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV146" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW146" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX146" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY146" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ146" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA146" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB146" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC146" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N147" t="n">
+        <v>10</v>
+      </c>
+      <c r="O147" t="n">
+        <v>10</v>
+      </c>
+      <c r="R147" t="n">
+        <v>0.004682466352329423</v>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA147" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO147" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP147" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ147" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS147" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT147" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU147" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV147" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW147" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX147" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY147" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ147" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA147" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB147" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC147" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N148" t="n">
+        <v>10</v>
+      </c>
+      <c r="O148" t="n">
+        <v>10</v>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W148" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X148" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z148" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA148" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC148" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD148" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE148" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF148" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG148" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH148" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI148" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ148" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK148" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM148" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN148" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO148" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP148" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ148" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS148" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT148" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU148" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV148" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW148" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX148" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY148" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ148" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA148" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB148" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC148" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>D021</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Dengue</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>登革热</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N149" t="n">
+        <v>4484</v>
+      </c>
+      <c r="O149" t="n">
+        <v>4484</v>
+      </c>
+      <c r="R149" t="n">
+        <v>2.099617912384513</v>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO149" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP149" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR149" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS149" t="inlineStr"/>
+      <c r="AT149" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU149" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV149" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW149" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX149" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY149" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ149" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA149" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB149" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC149" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>D052</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Chikungunya</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>基孔肯雅热</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N150" t="n">
+        <v>451</v>
+      </c>
+      <c r="O150" t="n">
+        <v>451</v>
+      </c>
+      <c r="R150" t="n">
+        <v>0.211179232490057</v>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO150" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP150" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR150" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS150" t="inlineStr"/>
+      <c r="AT150" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU150" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV150" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW150" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX150" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY150" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ150" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA150" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB150" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC150" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -22144,7 +24296,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
@@ -22154,7 +24306,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>137</v>
+        <v>149</v>
       </c>
     </row>
     <row r="11">
@@ -22174,7 +24326,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -22206,7 +24358,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1109933</v>
+        <v>1112400</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-26 04:01:59 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">
@@ -18409,13 +18409,13 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>40512</v>
+        <v>39691</v>
       </c>
       <c r="O115" t="n">
-        <v>40512</v>
+        <v>39691</v>
       </c>
       <c r="R115" t="n">
-        <v>18.96960768655696</v>
+        <v>18.58517719903071</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -18554,13 +18554,13 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="O116" t="n">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="R116" t="n">
-        <v>0.1493706766393086</v>
+        <v>0.1563943761678027</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -18989,13 +18989,13 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1490</v>
+        <v>1539</v>
       </c>
       <c r="O119" t="n">
-        <v>1490</v>
+        <v>1539</v>
       </c>
       <c r="R119" t="n">
-        <v>0.697687486497084</v>
+        <v>0.7206315716234982</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -19134,13 +19134,13 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>11782</v>
+        <v>11872</v>
       </c>
       <c r="O120" t="n">
-        <v>11782</v>
+        <v>11872</v>
       </c>
       <c r="R120" t="n">
-        <v>5.516881856314526</v>
+        <v>5.559024053485491</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -19424,13 +19424,13 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="O122" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="R122" t="n">
-        <v>0.03745973081863539</v>
+        <v>0.03792797745386832</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
@@ -19569,13 +19569,13 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="O123" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="R123" t="n">
-        <v>0.01779337213885181</v>
+        <v>0.02388057839688006</v>
       </c>
       <c r="S123" t="inlineStr">
         <is>
@@ -19714,13 +19714,13 @@
         </is>
       </c>
       <c r="N124" t="n">
-        <v>26801</v>
+        <v>31413</v>
       </c>
       <c r="O124" t="n">
-        <v>26801</v>
+        <v>31413</v>
       </c>
       <c r="R124" t="n">
-        <v>12.54947807087809</v>
+        <v>14.70903155257242</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
@@ -20825,7 +20825,7 @@
       </c>
       <c r="AJ131" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK131" t="inlineStr">
@@ -21218,7 +21218,7 @@
       </c>
       <c r="AJ133" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
         </is>
       </c>
       <c r="AK133" t="inlineStr">
@@ -21660,13 +21660,13 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>1597</v>
+        <v>2623</v>
       </c>
       <c r="O136" t="n">
-        <v>1597</v>
+        <v>2623</v>
       </c>
       <c r="R136" t="n">
-        <v>0.7477898764670088</v>
+        <v>1.228210924216008</v>
       </c>
       <c r="S136" t="inlineStr">
         <is>
@@ -21819,10 +21819,10 @@
         </is>
       </c>
       <c r="N137" t="n">
-        <v>1597</v>
+        <v>2623</v>
       </c>
       <c r="O137" t="n">
-        <v>1597</v>
+        <v>2623</v>
       </c>
       <c r="U137" t="inlineStr">
         <is>
@@ -22053,13 +22053,13 @@
         </is>
       </c>
       <c r="N138" t="n">
-        <v>38015</v>
+        <v>35953</v>
       </c>
       <c r="O138" t="n">
-        <v>38015</v>
+        <v>35953</v>
       </c>
       <c r="R138" t="n">
-        <v>17.8003958383803</v>
+        <v>16.83487127652997</v>
       </c>
       <c r="S138" t="inlineStr">
         <is>
@@ -22198,13 +22198,13 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>132</v>
+        <v>237</v>
       </c>
       <c r="O139" t="n">
-        <v>132</v>
+        <v>237</v>
       </c>
       <c r="R139" t="n">
-        <v>0.06180855585074838</v>
+        <v>0.1109744525502073</v>
       </c>
       <c r="S139" t="inlineStr">
         <is>
@@ -22314,22 +22314,22 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -22343,13 +22343,13 @@
         </is>
       </c>
       <c r="N140" t="n">
-        <v>723</v>
+        <v>1</v>
       </c>
       <c r="O140" t="n">
-        <v>723</v>
+        <v>1</v>
       </c>
       <c r="R140" t="n">
-        <v>0.3385423172734173</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S140" t="inlineStr">
         <is>
@@ -22459,17 +22459,17 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -22488,13 +22488,13 @@
         </is>
       </c>
       <c r="N141" t="n">
-        <v>8213</v>
+        <v>870</v>
       </c>
       <c r="O141" t="n">
-        <v>8213</v>
+        <v>870</v>
       </c>
       <c r="R141" t="n">
-        <v>3.845709615168155</v>
+        <v>0.4073745726526597</v>
       </c>
       <c r="S141" t="inlineStr">
         <is>
@@ -22604,22 +22604,22 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -22633,13 +22633,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>24</v>
+        <v>8691</v>
       </c>
       <c r="O142" t="n">
-        <v>24</v>
+        <v>8691</v>
       </c>
       <c r="R142" t="n">
-        <v>0.01123791924559061</v>
+        <v>4.069531506809501</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -22749,22 +22749,22 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -22778,13 +22778,13 @@
         </is>
       </c>
       <c r="N143" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="O143" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="R143" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.03418200437200478</v>
       </c>
       <c r="S143" t="inlineStr">
         <is>
@@ -22894,17 +22894,17 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -22923,13 +22923,13 @@
         </is>
       </c>
       <c r="N144" t="n">
-        <v>2970</v>
+        <v>31</v>
       </c>
       <c r="O144" t="n">
-        <v>2970</v>
+        <v>31</v>
       </c>
       <c r="R144" t="n">
-        <v>1.390692506641839</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S144" t="inlineStr">
         <is>
@@ -23039,17 +23039,17 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>D185</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Work accident with biological material</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>生物材料职业暴露事故</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -23068,13 +23068,13 @@
         </is>
       </c>
       <c r="N145" t="n">
-        <v>1855</v>
+        <v>29824</v>
       </c>
       <c r="O145" t="n">
-        <v>1855</v>
+        <v>29824</v>
       </c>
       <c r="R145" t="n">
-        <v>0.8685975083571079</v>
+        <v>13.96498764918727</v>
       </c>
       <c r="S145" t="inlineStr">
         <is>
@@ -23184,17 +23184,17 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>D186</t>
+          <t>D185</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Serious work accident</t>
+          <t>Work accident with biological material</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>严重工伤</t>
+          <t>生物材料职业暴露事故</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -23213,13 +23213,13 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>12573</v>
+        <v>1855</v>
       </c>
       <c r="O146" t="n">
-        <v>12573</v>
+        <v>1855</v>
       </c>
       <c r="R146" t="n">
-        <v>5.887264944783783</v>
+        <v>0.8685975083571079</v>
       </c>
       <c r="S146" t="inlineStr">
         <is>
@@ -23329,17 +23329,17 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>D188</t>
+          <t>D186</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Work-related cancer</t>
+          <t>Serious work accident</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>职业相关癌症</t>
+          <t>严重工伤</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -23358,13 +23358,13 @@
         </is>
       </c>
       <c r="N147" t="n">
-        <v>31</v>
+        <v>12573</v>
       </c>
       <c r="O147" t="n">
-        <v>31</v>
+        <v>12573</v>
       </c>
       <c r="R147" t="n">
-        <v>0.01451564569222121</v>
+        <v>5.887264944783783</v>
       </c>
       <c r="S147" t="inlineStr">
         <is>
@@ -23474,17 +23474,17 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>D189</t>
+          <t>D188</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Work-related dermatosis</t>
+          <t>Work-related cancer</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>职业性皮肤病</t>
+          <t>职业相关癌症</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -23503,13 +23503,13 @@
         </is>
       </c>
       <c r="N148" t="n">
-        <v>123</v>
+        <v>31</v>
       </c>
       <c r="O148" t="n">
-        <v>123</v>
+        <v>31</v>
       </c>
       <c r="R148" t="n">
-        <v>0.0575943361336519</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S148" t="inlineStr">
         <is>
@@ -23619,17 +23619,17 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>D192</t>
+          <t>D189</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Work-related repetitive strain injury</t>
+          <t>Work-related dermatosis</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>职业相关重复性劳损</t>
+          <t>职业性皮肤病</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -23648,55 +23648,41 @@
         </is>
       </c>
       <c r="N149" t="n">
-        <v>391</v>
+        <v>123</v>
       </c>
       <c r="O149" t="n">
-        <v>391</v>
+        <v>123</v>
       </c>
       <c r="R149" t="n">
-        <v>0.1830844343760804</v>
+        <v>0.0575943361336519</v>
       </c>
       <c r="S149" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
-      <c r="AA149" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO149" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP149" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ149" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS149" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR149" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS149" t="inlineStr"/>
       <c r="AT149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU149" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV149" t="inlineStr">
@@ -23763,7 +23749,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -23812,98 +23798,23 @@
       <c r="O150" t="n">
         <v>391</v>
       </c>
+      <c r="R150" t="n">
+        <v>0.1830844343760804</v>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U150" t="inlineStr">
         <is>
           <t>SER_BR_LERD</t>
         </is>
       </c>
-      <c r="V150" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
-      <c r="W150" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X150" t="inlineStr">
-        <is>
-          <t>Work-related repetitive strain injury</t>
-        </is>
-      </c>
-      <c r="Y150" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z150" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA150" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB150" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC150" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD150" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE150" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF150" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG150" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH150" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI150" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ150" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
-        </is>
-      </c>
-      <c r="AK150" t="inlineStr">
-        <is>
-          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
-        </is>
-      </c>
-      <c r="AM150" t="inlineStr">
-        <is>
-          <t>final; provisional</t>
-        </is>
-      </c>
-      <c r="AN150" t="b">
-        <v>1</v>
       </c>
       <c r="AO150" t="inlineStr">
         <is>
@@ -23997,7 +23908,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -24012,17 +23923,17 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>D193</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Work-related mental disorder</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>职业相关精神障碍</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -24041,22 +23952,39 @@
         </is>
       </c>
       <c r="N151" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="O151" t="n">
-        <v>172</v>
-      </c>
-      <c r="R151" t="n">
-        <v>0.08053842126006606</v>
-      </c>
-      <c r="S151" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>391</v>
       </c>
       <c r="U151" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>SER_BR_LERD</t>
+        </is>
+      </c>
+      <c r="W151" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X151" t="inlineStr">
+        <is>
+          <t>Work-related repetitive strain injury</t>
+        </is>
+      </c>
+      <c r="Y151" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z151" t="inlineStr">
+        <is>
+          <t>notification</t>
         </is>
       </c>
       <c r="AA151" t="inlineStr">
@@ -24064,6 +23992,64 @@
           <t>monthly</t>
         </is>
       </c>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC151" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD151" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE151" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF151" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG151" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH151" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI151" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ151" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
+        </is>
+      </c>
+      <c r="AK151" t="inlineStr">
+        <is>
+          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
+        </is>
+      </c>
+      <c r="AM151" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN151" t="b">
+        <v>1</v>
+      </c>
       <c r="AO151" t="inlineStr">
         <is>
           <t>series_registry</t>
@@ -24081,7 +24067,7 @@
       </c>
       <c r="AS151" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT151" t="n">
@@ -24156,7 +24142,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -24205,98 +24191,23 @@
       <c r="O152" t="n">
         <v>172</v>
       </c>
+      <c r="R152" t="n">
+        <v>0.08053842126006606</v>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U152" t="inlineStr">
         <is>
           <t>SER_BR_WORK_MENTAL_MENT</t>
         </is>
       </c>
-      <c r="V152" t="inlineStr">
-        <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
-        </is>
-      </c>
-      <c r="W152" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X152" t="inlineStr">
-        <is>
-          <t>Work-related mental disorder</t>
-        </is>
-      </c>
-      <c r="Y152" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z152" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA152" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB152" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC152" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD152" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE152" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF152" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG152" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH152" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI152" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ152" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.08.30.1</t>
-        </is>
-      </c>
-      <c r="AK152" t="inlineStr">
-        <is>
-          <t>SINAN MENT work-related mental disorder notifications.</t>
-        </is>
-      </c>
-      <c r="AM152" t="inlineStr">
-        <is>
-          <t>final; provisional</t>
-        </is>
-      </c>
-      <c r="AN152" t="b">
-        <v>1</v>
       </c>
       <c r="AO152" t="inlineStr">
         <is>
@@ -24390,7 +24301,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -24405,17 +24316,17 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>D194</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Noise-induced hearing loss</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>噪声性听力损失</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -24434,41 +24345,130 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="O153" t="n">
-        <v>14</v>
-      </c>
-      <c r="R153" t="n">
-        <v>0.006555452893261191</v>
-      </c>
-      <c r="S153" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>172</v>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="W153" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X153" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="Y153" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z153" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA153" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB153" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC153" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD153" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE153" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF153" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG153" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH153" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI153" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ153" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
+        </is>
+      </c>
+      <c r="AK153" t="inlineStr">
+        <is>
+          <t>SINAN MENT work-related mental disorder notifications.</t>
+        </is>
+      </c>
+      <c r="AM153" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN153" t="b">
+        <v>1</v>
       </c>
       <c r="AO153" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP153" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR153" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS153" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ153" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS153" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU153" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV153" t="inlineStr">
@@ -24550,17 +24550,17 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>D195</t>
+          <t>D194</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Pneumoconiosis</t>
+          <t>Noise-induced hearing loss</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>尘肺病</t>
+          <t>噪声性听力损失</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -24579,13 +24579,13 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="O154" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="R154" t="n">
-        <v>0.003277726446630596</v>
+        <v>0.006555452893261191</v>
       </c>
       <c r="S154" t="inlineStr">
         <is>
@@ -24695,17 +24695,17 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D195</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Pneumoconiosis</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>尘肺病</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -24724,55 +24724,41 @@
         </is>
       </c>
       <c r="N155" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="O155" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="R155" t="n">
-        <v>0.004682466352329423</v>
+        <v>0.003277726446630596</v>
       </c>
       <c r="S155" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA155" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO155" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP155" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ155" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS155" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR155" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS155" t="inlineStr"/>
       <c r="AT155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU155" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV155" t="inlineStr">
@@ -24839,7 +24825,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -24883,103 +24869,28 @@
         </is>
       </c>
       <c r="N156" t="n">
-        <v>10</v>
+        <v>2173</v>
       </c>
       <c r="O156" t="n">
-        <v>10</v>
+        <v>2173</v>
+      </c>
+      <c r="R156" t="n">
+        <v>1.017499938361184</v>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="U156" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V156" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W156" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X156" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y156" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z156" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA156" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB156" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC156" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD156" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE156" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF156" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG156" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH156" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI156" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ156" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK156" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM156" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN156" t="b">
-        <v>1</v>
       </c>
       <c r="AO156" t="inlineStr">
         <is>
@@ -25073,7 +24984,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -25088,70 +24999,159 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N157" t="n">
-        <v>11319</v>
+        <v>2173</v>
       </c>
       <c r="O157" t="n">
-        <v>11319</v>
-      </c>
-      <c r="R157" t="n">
-        <v>5.300083664201673</v>
-      </c>
-      <c r="S157" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>2173</v>
+      </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W157" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X157" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y157" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z157" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA157" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB157" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC157" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD157" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE157" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF157" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG157" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH157" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI157" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ157" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK157" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM157" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN157" t="b">
+        <v>1</v>
       </c>
       <c r="AO157" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP157" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR157" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS157" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ157" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS157" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU157" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV157" t="inlineStr">
@@ -25233,22 +25233,22 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L158" t="inlineStr">
@@ -25262,13 +25262,13 @@
         </is>
       </c>
       <c r="N158" t="n">
-        <v>1</v>
+        <v>19662</v>
       </c>
       <c r="O158" t="n">
-        <v>1</v>
+        <v>19662</v>
       </c>
       <c r="R158" t="n">
-        <v>0.0004682466352329422</v>
+        <v>9.20666534195011</v>
       </c>
       <c r="S158" t="inlineStr">
         <is>
@@ -25378,22 +25378,22 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
@@ -25407,13 +25407,13 @@
         </is>
       </c>
       <c r="N159" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="O159" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="R159" t="n">
-        <v>0.007491946163727075</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S159" t="inlineStr">
         <is>
@@ -25523,22 +25523,22 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
@@ -25552,13 +25552,13 @@
         </is>
       </c>
       <c r="N160" t="n">
-        <v>1384</v>
+        <v>1</v>
       </c>
       <c r="O160" t="n">
-        <v>1384</v>
+        <v>1</v>
       </c>
       <c r="R160" t="n">
-        <v>0.648053343162392</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S160" t="inlineStr">
         <is>
@@ -25625,6 +25625,1124 @@
         </is>
       </c>
       <c r="BC160" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>D051</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Zika virus disease</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>寨卡病毒病</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>59</v>
+      </c>
+      <c r="O161" t="n">
+        <v>59</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0.02762655147874359</v>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO161" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP161" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR161" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS161" t="inlineStr"/>
+      <c r="AT161" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU161" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV161" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW161" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX161" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY161" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ161" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA161" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB161" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC161" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>D052</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Chikungunya</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>基孔肯雅热</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>2846</v>
+      </c>
+      <c r="O162" t="n">
+        <v>2846</v>
+      </c>
+      <c r="R162" t="n">
+        <v>1.332629923872954</v>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO162" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP162" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR162" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS162" t="inlineStr"/>
+      <c r="AT162" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU162" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV162" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW162" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX162" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY162" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ162" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA162" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB162" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC162" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>5</v>
+      </c>
+      <c r="O163" t="n">
+        <v>5</v>
+      </c>
+      <c r="R163" t="n">
+        <v>0.002341233176164712</v>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO163" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP163" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR163" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS163" t="inlineStr"/>
+      <c r="AT163" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU163" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV163" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW163" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX163" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY163" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ163" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA163" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB163" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC163" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>D178</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Acute flaccid paralysis</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>急性无力肢体麻痹</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>7</v>
+      </c>
+      <c r="O164" t="n">
+        <v>7</v>
+      </c>
+      <c r="R164" t="n">
+        <v>0.003277726446630596</v>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO164" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP164" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR164" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS164" t="inlineStr"/>
+      <c r="AT164" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU164" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV164" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW164" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX164" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY164" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ164" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA164" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB164" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC164" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>D184</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Accident caused by venomous animals</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>毒性动物伤害</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>1082</v>
+      </c>
+      <c r="O165" t="n">
+        <v>1082</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0.5066428593220436</v>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO165" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP165" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR165" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS165" t="inlineStr"/>
+      <c r="AT165" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU165" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV165" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW165" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX165" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY165" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ165" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA165" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB165" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC165" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>357</v>
+      </c>
+      <c r="O166" t="n">
+        <v>357</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0.1671640487781604</v>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA166" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO166" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP166" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ166" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS166" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT166" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU166" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV166" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW166" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX166" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY166" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ166" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA166" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB166" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC166" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>357</v>
+      </c>
+      <c r="O167" t="n">
+        <v>357</v>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W167" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X167" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y167" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z167" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB167" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC167" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD167" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE167" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF167" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG167" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH167" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI167" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ167" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK167" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM167" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN167" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO167" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP167" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ167" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS167" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT167" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU167" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY167" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC167" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -25746,7 +26864,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>143</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
@@ -25756,7 +26874,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>159</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11">
@@ -25776,7 +26894,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -25808,7 +26926,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1184928</v>
+        <v>1229008</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-05 15:04:34 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -21631,22 +21631,22 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D201</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exanthematous diseases</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>出疹性疾病</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L136" t="inlineStr">
@@ -21660,55 +21660,41 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2623</v>
+        <v>439</v>
       </c>
       <c r="O136" t="n">
-        <v>2623</v>
+        <v>439</v>
       </c>
       <c r="R136" t="n">
-        <v>1.228210924216008</v>
+        <v>0.2055602728672617</v>
       </c>
       <c r="S136" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA136" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO136" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP136" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ136" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS136" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR136" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS136" t="inlineStr"/>
       <c r="AT136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU136" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV136" t="inlineStr">
@@ -21775,7 +21761,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -21824,98 +21810,23 @@
       <c r="O137" t="n">
         <v>2623</v>
       </c>
+      <c r="R137" t="n">
+        <v>1.228210924216008</v>
+      </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U137" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V137" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W137" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X137" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y137" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z137" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA137" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB137" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC137" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD137" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE137" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF137" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG137" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH137" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI137" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ137" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK137" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM137" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN137" t="b">
-        <v>1</v>
       </c>
       <c r="AO137" t="inlineStr">
         <is>
@@ -22009,7 +21920,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -22024,70 +21935,159 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N138" t="n">
-        <v>35953</v>
+        <v>2623</v>
       </c>
       <c r="O138" t="n">
-        <v>35953</v>
-      </c>
-      <c r="R138" t="n">
-        <v>16.83487127652997</v>
-      </c>
-      <c r="S138" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>2623</v>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W138" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X138" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z138" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA138" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC138" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD138" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE138" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF138" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG138" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH138" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI138" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ138" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK138" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM138" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN138" t="b">
+        <v>1</v>
       </c>
       <c r="AO138" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP138" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR138" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS138" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ138" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS138" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU138" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV138" t="inlineStr">
@@ -22169,22 +22169,22 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
@@ -22198,13 +22198,13 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>237</v>
+        <v>34742</v>
       </c>
       <c r="O139" t="n">
-        <v>237</v>
+        <v>34742</v>
       </c>
       <c r="R139" t="n">
-        <v>0.1109744525502073</v>
+        <v>16.26782460126288</v>
       </c>
       <c r="S139" t="inlineStr">
         <is>
@@ -22314,17 +22314,17 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -22343,13 +22343,13 @@
         </is>
       </c>
       <c r="N140" t="n">
-        <v>1</v>
+        <v>237</v>
       </c>
       <c r="O140" t="n">
-        <v>1</v>
+        <v>237</v>
       </c>
       <c r="R140" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.1109744525502073</v>
       </c>
       <c r="S140" t="inlineStr">
         <is>
@@ -22459,22 +22459,22 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">
@@ -22488,13 +22488,13 @@
         </is>
       </c>
       <c r="N141" t="n">
-        <v>870</v>
+        <v>1</v>
       </c>
       <c r="O141" t="n">
-        <v>870</v>
+        <v>1</v>
       </c>
       <c r="R141" t="n">
-        <v>0.4073745726526597</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S141" t="inlineStr">
         <is>
@@ -22604,22 +22604,22 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D042</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Leprosy</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>麻风病</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
@@ -22633,13 +22633,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>8691</v>
+        <v>1500</v>
       </c>
       <c r="O142" t="n">
-        <v>8691</v>
+        <v>1500</v>
       </c>
       <c r="R142" t="n">
-        <v>4.069531506809501</v>
+        <v>0.7023699528494134</v>
       </c>
       <c r="S142" t="inlineStr">
         <is>
@@ -22749,22 +22749,22 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -22778,13 +22778,13 @@
         </is>
       </c>
       <c r="N143" t="n">
-        <v>73</v>
+        <v>990</v>
       </c>
       <c r="O143" t="n">
-        <v>73</v>
+        <v>990</v>
       </c>
       <c r="R143" t="n">
-        <v>0.03418200437200478</v>
+        <v>0.4635641688806129</v>
       </c>
       <c r="S143" t="inlineStr">
         <is>
@@ -22894,22 +22894,22 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L144" t="inlineStr">
@@ -22923,13 +22923,13 @@
         </is>
       </c>
       <c r="N144" t="n">
-        <v>31</v>
+        <v>8912</v>
       </c>
       <c r="O144" t="n">
-        <v>31</v>
+        <v>8912</v>
       </c>
       <c r="R144" t="n">
-        <v>0.01451564569222121</v>
+        <v>4.173014013195981</v>
       </c>
       <c r="S144" t="inlineStr">
         <is>
@@ -23039,22 +23039,22 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L145" t="inlineStr">
@@ -23068,13 +23068,13 @@
         </is>
       </c>
       <c r="N145" t="n">
-        <v>29824</v>
+        <v>73</v>
       </c>
       <c r="O145" t="n">
-        <v>29824</v>
+        <v>73</v>
       </c>
       <c r="R145" t="n">
-        <v>13.96498764918727</v>
+        <v>0.03418200437200478</v>
       </c>
       <c r="S145" t="inlineStr">
         <is>
@@ -23184,17 +23184,17 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>D185</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Work accident with biological material</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>生物材料职业暴露事故</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -23213,13 +23213,13 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>1855</v>
+        <v>31</v>
       </c>
       <c r="O146" t="n">
-        <v>1855</v>
+        <v>31</v>
       </c>
       <c r="R146" t="n">
-        <v>0.8685975083571079</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S146" t="inlineStr">
         <is>
@@ -23329,17 +23329,17 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>D186</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Serious work accident</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>严重工伤</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -23358,13 +23358,13 @@
         </is>
       </c>
       <c r="N147" t="n">
-        <v>12573</v>
+        <v>29824</v>
       </c>
       <c r="O147" t="n">
-        <v>12573</v>
+        <v>29824</v>
       </c>
       <c r="R147" t="n">
-        <v>5.887264944783783</v>
+        <v>13.96498764918727</v>
       </c>
       <c r="S147" t="inlineStr">
         <is>
@@ -23474,17 +23474,17 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>D188</t>
+          <t>D185</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Work-related cancer</t>
+          <t>Work accident with biological material</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>职业相关癌症</t>
+          <t>生物材料职业暴露事故</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -23503,13 +23503,13 @@
         </is>
       </c>
       <c r="N148" t="n">
-        <v>31</v>
+        <v>1855</v>
       </c>
       <c r="O148" t="n">
-        <v>31</v>
+        <v>1855</v>
       </c>
       <c r="R148" t="n">
-        <v>0.01451564569222121</v>
+        <v>0.8685975083571079</v>
       </c>
       <c r="S148" t="inlineStr">
         <is>
@@ -23619,17 +23619,17 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>D189</t>
+          <t>D186</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Work-related dermatosis</t>
+          <t>Serious work accident</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>职业性皮肤病</t>
+          <t>严重工伤</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -23648,13 +23648,13 @@
         </is>
       </c>
       <c r="N149" t="n">
-        <v>123</v>
+        <v>12573</v>
       </c>
       <c r="O149" t="n">
-        <v>123</v>
+        <v>12573</v>
       </c>
       <c r="R149" t="n">
-        <v>0.0575943361336519</v>
+        <v>5.887264944783783</v>
       </c>
       <c r="S149" t="inlineStr">
         <is>
@@ -23764,17 +23764,17 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>D192</t>
+          <t>D188</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Work-related repetitive strain injury</t>
+          <t>Work-related cancer</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>职业相关重复性劳损</t>
+          <t>职业相关癌症</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -23793,55 +23793,41 @@
         </is>
       </c>
       <c r="N150" t="n">
-        <v>391</v>
+        <v>31</v>
       </c>
       <c r="O150" t="n">
-        <v>391</v>
+        <v>31</v>
       </c>
       <c r="R150" t="n">
-        <v>0.1830844343760804</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S150" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
-      <c r="AA150" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO150" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP150" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ150" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS150" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR150" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS150" t="inlineStr"/>
       <c r="AT150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU150" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV150" t="inlineStr">
@@ -23908,7 +23894,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -23923,17 +23909,17 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>D192</t>
+          <t>D189</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Work-related repetitive strain injury</t>
+          <t>Work-related dermatosis</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>职业相关重复性劳损</t>
+          <t>职业性皮肤病</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -23952,130 +23938,41 @@
         </is>
       </c>
       <c r="N151" t="n">
-        <v>391</v>
+        <v>123</v>
       </c>
       <c r="O151" t="n">
-        <v>391</v>
-      </c>
-      <c r="U151" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
-      <c r="V151" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
-      <c r="W151" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X151" t="inlineStr">
-        <is>
-          <t>Work-related repetitive strain injury</t>
-        </is>
-      </c>
-      <c r="Y151" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z151" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="AA151" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB151" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC151" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD151" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE151" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF151" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AG151" t="inlineStr">
-        <is>
-          <t>non_additive</t>
-        </is>
-      </c>
-      <c r="AH151" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI151" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ151" t="inlineStr">
-        <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
-        </is>
-      </c>
-      <c r="AK151" t="inlineStr">
-        <is>
-          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
-        </is>
-      </c>
-      <c r="AM151" t="inlineStr">
-        <is>
-          <t>final; provisional</t>
-        </is>
-      </c>
-      <c r="AN151" t="b">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="R151" t="n">
+        <v>0.0575943361336519</v>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="AO151" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP151" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ151" t="inlineStr">
-        <is>
-          <t>parity</t>
-        </is>
-      </c>
-      <c r="AS151" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR151" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS151" t="inlineStr"/>
       <c r="AT151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU151" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV151" t="inlineStr">
@@ -24157,17 +24054,17 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>D193</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Work-related mental disorder</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>职业相关精神障碍</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -24186,13 +24083,13 @@
         </is>
       </c>
       <c r="N152" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="O152" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="R152" t="n">
-        <v>0.08053842126006606</v>
+        <v>0.1830844343760804</v>
       </c>
       <c r="S152" t="inlineStr">
         <is>
@@ -24201,7 +24098,7 @@
       </c>
       <c r="U152" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AA152" t="inlineStr">
@@ -24226,7 +24123,7 @@
       </c>
       <c r="AS152" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT152" t="n">
@@ -24316,17 +24213,17 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>D193</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Work-related mental disorder</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>职业相关精神障碍</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -24345,19 +24242,19 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="O153" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="U153" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="V153" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="W153" t="inlineStr">
@@ -24367,7 +24264,7 @@
       </c>
       <c r="X153" t="inlineStr">
         <is>
-          <t>Work-related mental disorder</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="Y153" t="inlineStr">
@@ -24432,7 +24329,7 @@
       </c>
       <c r="AK153" t="inlineStr">
         <is>
-          <t>SINAN MENT work-related mental disorder notifications.</t>
+          <t>SINAN LERD work-related repetitive strain injury or musculoskeletal disorder notifications; LER is retained as the historical source code alias.</t>
         </is>
       </c>
       <c r="AM153" t="inlineStr">
@@ -24460,7 +24357,7 @@
       </c>
       <c r="AS153" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT153" t="n">
@@ -24550,17 +24447,17 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>D194</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Noise-induced hearing loss</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>噪声性听力损失</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -24579,41 +24476,55 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="O154" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="R154" t="n">
-        <v>0.006555452893261191</v>
+        <v>0.08053842126006606</v>
       </c>
       <c r="S154" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="AA154" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO154" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP154" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR154" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS154" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ154" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS154" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU154" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV154" t="inlineStr">
@@ -24680,7 +24591,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -24695,17 +24606,17 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>D195</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Pneumoconiosis</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>尘肺病</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
@@ -24724,41 +24635,130 @@
         </is>
       </c>
       <c r="N155" t="n">
-        <v>7</v>
+        <v>172</v>
       </c>
       <c r="O155" t="n">
-        <v>7</v>
-      </c>
-      <c r="R155" t="n">
-        <v>0.003277726446630596</v>
-      </c>
-      <c r="S155" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>172</v>
+      </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
+      <c r="W155" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X155" t="inlineStr">
+        <is>
+          <t>Work-related mental disorder</t>
+        </is>
+      </c>
+      <c r="Y155" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z155" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA155" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB155" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC155" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD155" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE155" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF155" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="AG155" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH155" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI155" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ155" t="inlineStr">
+        <is>
+          <t>globalid-disease-ontology:2026.09.26.1</t>
+        </is>
+      </c>
+      <c r="AK155" t="inlineStr">
+        <is>
+          <t>SINAN MENT work-related mental disorder notifications.</t>
+        </is>
+      </c>
+      <c r="AM155" t="inlineStr">
+        <is>
+          <t>final; provisional</t>
+        </is>
+      </c>
+      <c r="AN155" t="b">
+        <v>1</v>
       </c>
       <c r="AO155" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP155" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR155" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS155" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ155" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS155" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT155" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU155" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series.</t>
         </is>
       </c>
       <c r="AV155" t="inlineStr">
@@ -24840,17 +24840,17 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D194</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Noise-induced hearing loss</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>噪声性听力损失</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -24869,55 +24869,41 @@
         </is>
       </c>
       <c r="N156" t="n">
-        <v>2173</v>
+        <v>14</v>
       </c>
       <c r="O156" t="n">
-        <v>2173</v>
+        <v>14</v>
       </c>
       <c r="R156" t="n">
-        <v>1.017499938361184</v>
+        <v>0.006555452893261191</v>
       </c>
       <c r="S156" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA156" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO156" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP156" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ156" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS156" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR156" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS156" t="inlineStr"/>
       <c r="AT156" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU156" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV156" t="inlineStr">
@@ -24984,7 +24970,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -24999,17 +24985,17 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D195</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Pneumoconiosis</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>尘肺病</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -25028,130 +25014,41 @@
         </is>
       </c>
       <c r="N157" t="n">
-        <v>2173</v>
+        <v>7</v>
       </c>
       <c r="O157" t="n">
-        <v>2173</v>
-      </c>
-      <c r="U157" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="V157" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W157" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X157" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y157" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z157" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="AA157" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB157" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC157" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD157" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE157" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF157" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG157" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH157" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI157" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ157" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK157" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM157" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN157" t="b">
-        <v>1</v>
+        <v>7</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0.003277726446630596</v>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="AO157" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP157" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ157" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS157" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR157" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS157" t="inlineStr"/>
       <c r="AT157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU157" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV157" t="inlineStr">
@@ -25233,17 +25130,17 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D201</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Exanthematous diseases</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>出疹性疾病</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -25253,22 +25150,22 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N158" t="n">
-        <v>19662</v>
+        <v>2044</v>
       </c>
       <c r="O158" t="n">
-        <v>19662</v>
+        <v>2044</v>
       </c>
       <c r="R158" t="n">
-        <v>9.20666534195011</v>
+        <v>0.9570961224161341</v>
       </c>
       <c r="S158" t="inlineStr">
         <is>
@@ -25378,70 +25275,84 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N159" t="n">
-        <v>31</v>
+        <v>2173</v>
       </c>
       <c r="O159" t="n">
-        <v>31</v>
+        <v>2173</v>
       </c>
       <c r="R159" t="n">
-        <v>0.01451564569222121</v>
+        <v>1.017499938361184</v>
       </c>
       <c r="S159" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA159" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO159" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP159" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR159" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS159" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ159" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS159" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU159" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV159" t="inlineStr">
@@ -25508,7 +25419,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -25523,70 +25434,159 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N160" t="n">
+        <v>2173</v>
+      </c>
+      <c r="O160" t="n">
+        <v>2173</v>
+      </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W160" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X160" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y160" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z160" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA160" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB160" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC160" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD160" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE160" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF160" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG160" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH160" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI160" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ160" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK160" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM160" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN160" t="b">
         <v>1</v>
       </c>
-      <c r="O160" t="n">
+      <c r="AO160" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP160" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ160" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS160" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT160" t="n">
         <v>1</v>
       </c>
-      <c r="R160" t="n">
-        <v>0.0004682466352329422</v>
-      </c>
-      <c r="S160" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
-      </c>
-      <c r="AO160" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AP160" t="inlineStr">
-        <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR160" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS160" t="inlineStr"/>
-      <c r="AT160" t="n">
-        <v>0</v>
-      </c>
       <c r="AU160" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV160" t="inlineStr">
@@ -25668,17 +25668,17 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -25697,13 +25697,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>59</v>
+        <v>27095</v>
       </c>
       <c r="O161" t="n">
-        <v>59</v>
+        <v>27095</v>
       </c>
       <c r="R161" t="n">
-        <v>0.02762655147874359</v>
+        <v>12.68714258163657</v>
       </c>
       <c r="S161" t="inlineStr">
         <is>
@@ -25813,22 +25813,22 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L162" t="inlineStr">
@@ -25842,13 +25842,13 @@
         </is>
       </c>
       <c r="N162" t="n">
-        <v>2846</v>
+        <v>31</v>
       </c>
       <c r="O162" t="n">
-        <v>2846</v>
+        <v>31</v>
       </c>
       <c r="R162" t="n">
-        <v>1.332629923872954</v>
+        <v>0.01451564569222121</v>
       </c>
       <c r="S162" t="inlineStr">
         <is>
@@ -25958,17 +25958,17 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -25987,13 +25987,13 @@
         </is>
       </c>
       <c r="N163" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O163" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="R163" t="n">
-        <v>0.002341233176164712</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S163" t="inlineStr">
         <is>
@@ -26103,22 +26103,22 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D042</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Leprosy</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>麻风病</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L164" t="inlineStr">
@@ -26132,13 +26132,13 @@
         </is>
       </c>
       <c r="N164" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="O164" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="R164" t="n">
-        <v>0.003277726446630596</v>
+        <v>0.008896686069425903</v>
       </c>
       <c r="S164" t="inlineStr">
         <is>
@@ -26248,22 +26248,22 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -26277,13 +26277,13 @@
         </is>
       </c>
       <c r="N165" t="n">
-        <v>1082</v>
+        <v>183</v>
       </c>
       <c r="O165" t="n">
-        <v>1082</v>
+        <v>183</v>
       </c>
       <c r="R165" t="n">
-        <v>0.5066428593220436</v>
+        <v>0.08568913424762843</v>
       </c>
       <c r="S165" t="inlineStr">
         <is>
@@ -26393,22 +26393,22 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L166" t="inlineStr">
@@ -26422,55 +26422,41 @@
         </is>
       </c>
       <c r="N166" t="n">
-        <v>357</v>
+        <v>4420</v>
       </c>
       <c r="O166" t="n">
-        <v>357</v>
+        <v>4420</v>
       </c>
       <c r="R166" t="n">
-        <v>0.1671640487781604</v>
+        <v>2.069650127729605</v>
       </c>
       <c r="S166" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA166" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO166" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP166" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ166" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS166" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR166" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS166" t="inlineStr"/>
       <c r="AT166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU166" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV166" t="inlineStr">
@@ -26537,212 +26523,951 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>5</v>
+      </c>
+      <c r="O167" t="n">
+        <v>5</v>
+      </c>
+      <c r="R167" t="n">
+        <v>0.002341233176164712</v>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO167" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP167" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR167" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS167" t="inlineStr"/>
+      <c r="AT167" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU167" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY167" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC167" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>D178</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Acute flaccid paralysis</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>急性无力肢体麻痹</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>7</v>
+      </c>
+      <c r="O168" t="n">
+        <v>7</v>
+      </c>
+      <c r="R168" t="n">
+        <v>0.003277726446630596</v>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO168" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP168" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR168" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS168" t="inlineStr"/>
+      <c r="AT168" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU168" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV168" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW168" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX168" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY168" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ168" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA168" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB168" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC168" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>D184</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Accident caused by venomous animals</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>毒性动物伤害</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>1082</v>
+      </c>
+      <c r="O169" t="n">
+        <v>1082</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0.5066428593220436</v>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO169" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP169" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR169" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS169" t="inlineStr"/>
+      <c r="AT169" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU169" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV169" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW169" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX169" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY169" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ169" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA169" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB169" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC169" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>D201</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Exanthematous diseases</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>出疹性疾病</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>289</v>
+      </c>
+      <c r="O170" t="n">
+        <v>289</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0.1353232775823203</v>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO170" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP170" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR170" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS170" t="inlineStr"/>
+      <c r="AT170" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU170" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV170" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW170" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX170" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY170" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ170" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA170" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB170" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC170" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>357</v>
+      </c>
+      <c r="O171" t="n">
+        <v>357</v>
+      </c>
+      <c r="R171" t="n">
+        <v>0.1671640487781604</v>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA171" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO171" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP171" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ171" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS171" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT171" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU171" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV171" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW171" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX171" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY171" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ171" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA171" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB171" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC171" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
           <t>source_series_observation</t>
         </is>
       </c>
-      <c r="F167" t="inlineStr">
+      <c r="F172" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
         <is>
           <t>D235</t>
         </is>
       </c>
-      <c r="I167" t="inlineStr">
+      <c r="I172" t="inlineStr">
         <is>
           <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr">
+      <c r="J172" t="inlineStr">
         <is>
           <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr">
+      <c r="K172" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L167" t="inlineStr">
+      <c r="L172" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="M167" t="inlineStr">
+      <c r="M172" t="inlineStr">
         <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="N167" t="n">
+      <c r="N172" t="n">
         <v>357</v>
       </c>
-      <c r="O167" t="n">
+      <c r="O172" t="n">
         <v>357</v>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="U172" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V167" t="inlineStr">
+      <c r="V172" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="W167" t="inlineStr">
+      <c r="W172" t="inlineStr">
         <is>
           <t>SRC_BR_SINAN</t>
         </is>
       </c>
-      <c r="X167" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>Meningitis</t>
         </is>
       </c>
-      <c r="Y167" t="inlineStr">
+      <c r="Y172" t="inlineStr">
         <is>
           <t>case_notifications</t>
         </is>
       </c>
-      <c r="Z167" t="inlineStr">
+      <c r="Z172" t="inlineStr">
         <is>
           <t>notification</t>
         </is>
       </c>
-      <c r="AA167" t="inlineStr">
+      <c r="AA172" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="AB167" t="inlineStr">
+      <c r="AB172" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="AC167" t="inlineStr">
+      <c r="AC172" t="inlineStr">
         <is>
           <t>country:BR:national</t>
         </is>
       </c>
-      <c r="AD167" t="inlineStr">
+      <c r="AD172" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AE167" t="inlineStr">
+      <c r="AE172" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="AF167" t="inlineStr">
+      <c r="AF172" t="inlineStr">
         <is>
           <t>conditional</t>
         </is>
       </c>
-      <c r="AG167" t="inlineStr">
+      <c r="AG172" t="inlineStr">
         <is>
           <t>reported_aggregate</t>
         </is>
       </c>
-      <c r="AH167" t="inlineStr">
+      <c r="AH172" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="AI167" t="inlineStr">
+      <c r="AI172" t="inlineStr">
         <is>
           <t>missing_is_unknown</t>
         </is>
       </c>
-      <c r="AJ167" t="inlineStr">
+      <c r="AJ172" t="inlineStr">
         <is>
           <t>BR_SINAN_MENI_current</t>
         </is>
       </c>
-      <c r="AK167" t="inlineStr">
+      <c r="AK172" t="inlineStr">
         <is>
           <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
         </is>
       </c>
-      <c r="AM167" t="inlineStr">
+      <c r="AM172" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>
       </c>
-      <c r="AN167" t="b">
+      <c r="AN172" t="b">
         <v>1</v>
       </c>
-      <c r="AO167" t="inlineStr">
+      <c r="AO172" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="AP167" t="inlineStr">
+      <c r="AP172" t="inlineStr">
         <is>
           <t>single_series</t>
         </is>
       </c>
-      <c r="AQ167" t="inlineStr">
+      <c r="AQ172" t="inlineStr">
         <is>
           <t>legacy_gap_fill</t>
         </is>
       </c>
-      <c r="AS167" t="inlineStr">
+      <c r="AS172" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="AT167" t="n">
+      <c r="AT172" t="n">
         <v>1</v>
       </c>
-      <c r="AU167" t="inlineStr">
+      <c r="AU172" t="inlineStr">
         <is>
           <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
-      <c r="AV167" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="AW167" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="AX167" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="AY167" t="inlineStr">
-        <is>
-          <t>ftp_dbc</t>
-        </is>
-      </c>
-      <c r="AZ167" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="BA167" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="BB167" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="BC167" t="inlineStr">
+      <c r="AV172" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW172" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX172" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY172" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ172" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA172" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB172" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC172" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -26864,7 +27589,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10">
@@ -26874,7 +27599,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11">
@@ -26926,7 +27651,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1229008</v>
+        <v>1241560</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-21 16:13:09 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -19502,17 +19502,17 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>D188</t>
+          <t>D187</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Work-related cancer</t>
+          <t>Rabies post-exposure prophylaxis</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>职业相关癌症</t>
+          <t>狂犬病暴露后处置</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -19531,13 +19531,13 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>31</v>
+        <v>53431</v>
       </c>
       <c r="O139" t="n">
-        <v>31</v>
+        <v>53431</v>
       </c>
       <c r="R139" t="n">
-        <v>0.01447164822283888</v>
+        <v>24.94305278046788</v>
       </c>
       <c r="AA139" t="inlineStr">
         <is>
@@ -19637,17 +19637,17 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>D189</t>
+          <t>D188</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Work-related dermatosis</t>
+          <t>Work-related cancer</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>职业性皮肤病</t>
+          <t>职业相关癌症</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -19666,13 +19666,13 @@
         </is>
       </c>
       <c r="N140" t="n">
-        <v>123</v>
+        <v>31</v>
       </c>
       <c r="O140" t="n">
-        <v>123</v>
+        <v>31</v>
       </c>
       <c r="R140" t="n">
-        <v>0.05741976552932847</v>
+        <v>0.01447164822283888</v>
       </c>
       <c r="AA140" t="inlineStr">
         <is>
@@ -19772,17 +19772,17 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D189</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Work-related dermatosis</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>职业性皮肤病</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -19801,13 +19801,13 @@
         </is>
       </c>
       <c r="N141" t="n">
-        <v>24935</v>
+        <v>123</v>
       </c>
       <c r="O141" t="n">
-        <v>24935</v>
+        <v>123</v>
       </c>
       <c r="R141" t="n">
-        <v>11.64034027214476</v>
+        <v>0.05741976552932847</v>
       </c>
       <c r="AA141" t="inlineStr">
         <is>
@@ -19907,17 +19907,17 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>D192</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Work-related repetitive strain injury</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>职业相关重复性劳损</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -19936,18 +19936,13 @@
         </is>
       </c>
       <c r="N142" t="n">
-        <v>391</v>
+        <v>24935</v>
       </c>
       <c r="O142" t="n">
-        <v>391</v>
+        <v>24935</v>
       </c>
       <c r="R142" t="n">
-        <v>0.1825294985525808</v>
-      </c>
-      <c r="U142" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
+        <v>11.64034027214476</v>
       </c>
       <c r="AA142" t="inlineStr">
         <is>
@@ -19956,7 +19951,7 @@
       </c>
       <c r="AO142" t="inlineStr">
         <is>
-          <t>series_registry</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP142" t="inlineStr">
@@ -19964,13 +19959,9 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS142" t="inlineStr">
-        <is>
-          <t>SER_BR_LERD</t>
-        </is>
-      </c>
+      <c r="AS142" t="inlineStr"/>
       <c r="AT142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV142" t="inlineStr">
         <is>
@@ -20051,17 +20042,17 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>D193</t>
+          <t>D192</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Work-related mental disorder</t>
+          <t>Work-related repetitive strain injury</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>职业相关精神障碍</t>
+          <t>职业相关重复性劳损</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -20080,17 +20071,17 @@
         </is>
       </c>
       <c r="N143" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="O143" t="n">
-        <v>172</v>
+        <v>391</v>
       </c>
       <c r="R143" t="n">
-        <v>0.08029430626865444</v>
+        <v>0.1825294985525808</v>
       </c>
       <c r="U143" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AA143" t="inlineStr">
@@ -20110,7 +20101,7 @@
       </c>
       <c r="AS143" t="inlineStr">
         <is>
-          <t>SER_BR_WORK_MENTAL_MENT</t>
+          <t>SER_BR_LERD</t>
         </is>
       </c>
       <c r="AT143" t="n">
@@ -20195,17 +20186,17 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>D194</t>
+          <t>D193</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Noise-induced hearing loss</t>
+          <t>Work-related mental disorder</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>噪声性听力损失</t>
+          <t>职业相关精神障碍</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -20224,13 +20215,18 @@
         </is>
       </c>
       <c r="N144" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="O144" t="n">
-        <v>14</v>
+        <v>172</v>
       </c>
       <c r="R144" t="n">
-        <v>0.006535583068378851</v>
+        <v>0.08029430626865444</v>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
       </c>
       <c r="AA144" t="inlineStr">
         <is>
@@ -20239,7 +20235,7 @@
       </c>
       <c r="AO144" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>series_registry</t>
         </is>
       </c>
       <c r="AP144" t="inlineStr">
@@ -20247,9 +20243,13 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS144" t="inlineStr"/>
+      <c r="AS144" t="inlineStr">
+        <is>
+          <t>SER_BR_WORK_MENTAL_MENT</t>
+        </is>
+      </c>
       <c r="AT144" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV144" t="inlineStr">
         <is>
@@ -20330,17 +20330,17 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>D195</t>
+          <t>D194</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Pneumoconiosis</t>
+          <t>Noise-induced hearing loss</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>尘肺病</t>
+          <t>噪声性听力损失</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -20359,13 +20359,13 @@
         </is>
       </c>
       <c r="N145" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="O145" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="R145" t="n">
-        <v>0.003267791534189425</v>
+        <v>0.006535583068378851</v>
       </c>
       <c r="AA145" t="inlineStr">
         <is>
@@ -20465,22 +20465,22 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>D201</t>
+          <t>D195</t>
         </is>
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Exanthematous diseases</t>
+          <t>Pneumoconiosis</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>出疹性疾病</t>
+          <t>尘肺病</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L146" t="inlineStr">
@@ -20494,13 +20494,13 @@
         </is>
       </c>
       <c r="N146" t="n">
-        <v>2044</v>
+        <v>7</v>
       </c>
       <c r="O146" t="n">
-        <v>2044</v>
+        <v>7</v>
       </c>
       <c r="R146" t="n">
-        <v>0.9541951279833122</v>
+        <v>0.003267791534189425</v>
       </c>
       <c r="AA146" t="inlineStr">
         <is>
@@ -20600,22 +20600,22 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D201</t>
         </is>
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exanthematous diseases</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>出疹性疾病</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L147" t="inlineStr">
@@ -20629,18 +20629,13 @@
         </is>
       </c>
       <c r="N147" t="n">
-        <v>2173</v>
+        <v>2044</v>
       </c>
       <c r="O147" t="n">
-        <v>2173</v>
+        <v>2044</v>
       </c>
       <c r="R147" t="n">
-        <v>1.014415857684803</v>
-      </c>
-      <c r="U147" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
+        <v>0.9541951279833122</v>
       </c>
       <c r="AA147" t="inlineStr">
         <is>
@@ -20649,7 +20644,7 @@
       </c>
       <c r="AO147" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP147" t="inlineStr">
@@ -20657,13 +20652,9 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS147" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+      <c r="AS147" t="inlineStr"/>
       <c r="AT147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV147" t="inlineStr">
         <is>
@@ -20744,42 +20735,47 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N148" t="n">
-        <v>31476</v>
+        <v>2173</v>
       </c>
       <c r="O148" t="n">
-        <v>31476</v>
+        <v>2173</v>
       </c>
       <c r="R148" t="n">
-        <v>14.69385804716376</v>
+        <v>1.014415857684803</v>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
       </c>
       <c r="AA148" t="inlineStr">
         <is>
@@ -20788,7 +20784,7 @@
       </c>
       <c r="AO148" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP148" t="inlineStr">
@@ -20796,9 +20792,13 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS148" t="inlineStr"/>
+      <c r="AS148" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV148" t="inlineStr">
         <is>
@@ -20879,22 +20879,22 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
@@ -20908,13 +20908,13 @@
         </is>
       </c>
       <c r="N149" t="n">
-        <v>158</v>
+        <v>31476</v>
       </c>
       <c r="O149" t="n">
-        <v>158</v>
+        <v>31476</v>
       </c>
       <c r="R149" t="n">
-        <v>0.0737587232002756</v>
+        <v>14.69385804716376</v>
       </c>
       <c r="AA149" t="inlineStr">
         <is>
@@ -21014,17 +21014,17 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -21043,13 +21043,13 @@
         </is>
       </c>
       <c r="N150" t="n">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="O150" t="n">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="R150" t="n">
-        <v>0.0004668273620270607</v>
+        <v>0.0737587232002756</v>
       </c>
       <c r="AA150" t="inlineStr">
         <is>
@@ -21149,17 +21149,17 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>D042</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Leprosy</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>麻风病</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -21178,13 +21178,13 @@
         </is>
       </c>
       <c r="N151" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="O151" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="R151" t="n">
-        <v>0.008869719878514154</v>
+        <v>0.0004668273620270607</v>
       </c>
       <c r="AA151" t="inlineStr">
         <is>
@@ -21284,22 +21284,22 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D042</t>
         </is>
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Leprosy</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>麻风病</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L152" t="inlineStr">
@@ -21313,13 +21313,13 @@
         </is>
       </c>
       <c r="N152" t="n">
-        <v>425</v>
+        <v>19</v>
       </c>
       <c r="O152" t="n">
-        <v>425</v>
+        <v>19</v>
       </c>
       <c r="R152" t="n">
-        <v>0.1984016288615008</v>
+        <v>0.008869719878514154</v>
       </c>
       <c r="AA152" t="inlineStr">
         <is>
@@ -21419,17 +21419,17 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -21448,13 +21448,13 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>6782</v>
+        <v>425</v>
       </c>
       <c r="O153" t="n">
-        <v>6782</v>
+        <v>425</v>
       </c>
       <c r="R153" t="n">
-        <v>3.166023169267526</v>
+        <v>0.1984016288615008</v>
       </c>
       <c r="AA153" t="inlineStr">
         <is>
@@ -21554,17 +21554,17 @@
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>D054</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Varicella</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
         <is>
-          <t>水痘</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K154" t="inlineStr">
@@ -21583,13 +21583,13 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>610</v>
+        <v>6782</v>
       </c>
       <c r="O154" t="n">
-        <v>610</v>
+        <v>6782</v>
       </c>
       <c r="R154" t="n">
-        <v>0.2847646908365071</v>
+        <v>3.166023169267526</v>
       </c>
       <c r="AA154" t="inlineStr">
         <is>
@@ -21689,22 +21689,22 @@
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D054</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Varicella</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>水痘</t>
         </is>
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L155" t="inlineStr">
@@ -21718,13 +21718,13 @@
         </is>
       </c>
       <c r="N155" t="n">
-        <v>43</v>
+        <v>610</v>
       </c>
       <c r="O155" t="n">
-        <v>43</v>
+        <v>610</v>
       </c>
       <c r="R155" t="n">
-        <v>0.02007357656716361</v>
+        <v>0.2847646908365071</v>
       </c>
       <c r="AA155" t="inlineStr">
         <is>
@@ -21824,22 +21824,22 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>D168</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Congenital rubella syndrome</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>先天性风疹综合征</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L156" t="inlineStr">
@@ -21853,13 +21853,13 @@
         </is>
       </c>
       <c r="N156" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="O156" t="n">
-        <v>2</v>
+        <v>43</v>
       </c>
       <c r="R156" t="n">
-        <v>0.0009336547240541215</v>
+        <v>0.02007357656716361</v>
       </c>
       <c r="AA156" t="inlineStr">
         <is>
@@ -21959,22 +21959,22 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D168</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Congenital rubella syndrome</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>先天性风疹综合征</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
@@ -21988,13 +21988,13 @@
         </is>
       </c>
       <c r="N157" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O157" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="R157" t="n">
-        <v>0.003267791534189425</v>
+        <v>0.0009336547240541215</v>
       </c>
       <c r="AA157" t="inlineStr">
         <is>
@@ -22094,17 +22094,17 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K158" t="inlineStr">
@@ -22123,13 +22123,13 @@
         </is>
       </c>
       <c r="N158" t="n">
-        <v>1082</v>
+        <v>7</v>
       </c>
       <c r="O158" t="n">
-        <v>1082</v>
+        <v>7</v>
       </c>
       <c r="R158" t="n">
-        <v>0.5051072057132797</v>
+        <v>0.003267791534189425</v>
       </c>
       <c r="AA158" t="inlineStr">
         <is>
@@ -22229,17 +22229,17 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -22258,13 +22258,13 @@
         </is>
       </c>
       <c r="N159" t="n">
-        <v>5546</v>
+        <v>1082</v>
       </c>
       <c r="O159" t="n">
-        <v>5546</v>
+        <v>1082</v>
       </c>
       <c r="R159" t="n">
-        <v>2.589024549802079</v>
+        <v>0.5051072057132797</v>
       </c>
       <c r="AA159" t="inlineStr">
         <is>
@@ -22364,22 +22364,22 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>D201</t>
+          <t>D187</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Exanthematous diseases</t>
+          <t>Rabies post-exposure prophylaxis</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>出疹性疾病</t>
+          <t>狂犬病暴露后处置</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L160" t="inlineStr">
@@ -22393,13 +22393,13 @@
         </is>
       </c>
       <c r="N160" t="n">
-        <v>289</v>
+        <v>4434</v>
       </c>
       <c r="O160" t="n">
-        <v>289</v>
+        <v>4434</v>
       </c>
       <c r="R160" t="n">
-        <v>0.1349131076258205</v>
+        <v>2.069912523227988</v>
       </c>
       <c r="AA160" t="inlineStr">
         <is>
@@ -22499,17 +22499,17 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K161" t="inlineStr">
@@ -22528,18 +22528,13 @@
         </is>
       </c>
       <c r="N161" t="n">
-        <v>357</v>
+        <v>5546</v>
       </c>
       <c r="O161" t="n">
-        <v>357</v>
+        <v>5546</v>
       </c>
       <c r="R161" t="n">
-        <v>0.1666573682436607</v>
-      </c>
-      <c r="U161" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
+        <v>2.589024549802079</v>
       </c>
       <c r="AA161" t="inlineStr">
         <is>
@@ -22548,7 +22543,7 @@
       </c>
       <c r="AO161" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP161" t="inlineStr">
@@ -22556,13 +22551,9 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS161" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+      <c r="AS161" t="inlineStr"/>
       <c r="AT161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV161" t="inlineStr">
         <is>
@@ -22643,17 +22634,17 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D201</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Exanthematous diseases</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>出疹性疾病</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -22663,22 +22654,22 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="N162" t="n">
-        <v>9847</v>
+        <v>289</v>
       </c>
       <c r="O162" t="n">
-        <v>9847</v>
+        <v>289</v>
       </c>
       <c r="R162" t="n">
-        <v>4.596849033880467</v>
+        <v>0.1349131076258205</v>
       </c>
       <c r="AA162" t="inlineStr">
         <is>
@@ -22778,42 +22769,47 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="N163" t="n">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="O163" t="n">
-        <v>9</v>
+        <v>357</v>
       </c>
       <c r="R163" t="n">
-        <v>0.004201446258243547</v>
+        <v>0.1666573682436607</v>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
       </c>
       <c r="AA163" t="inlineStr">
         <is>
@@ -22822,7 +22818,7 @@
       </c>
       <c r="AO163" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP163" t="inlineStr">
@@ -22830,9 +22826,13 @@
           <t>published_series</t>
         </is>
       </c>
-      <c r="AS163" t="inlineStr"/>
+      <c r="AS163" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT163" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV163" t="inlineStr">
         <is>
@@ -22913,17 +22913,17 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -22942,13 +22942,13 @@
         </is>
       </c>
       <c r="N164" t="n">
-        <v>1079</v>
+        <v>9847</v>
       </c>
       <c r="O164" t="n">
-        <v>1079</v>
+        <v>9847</v>
       </c>
       <c r="R164" t="n">
-        <v>0.5037067236271986</v>
+        <v>4.596849033880467</v>
       </c>
       <c r="AA164" t="inlineStr">
         <is>
@@ -23048,22 +23048,22 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
@@ -23077,13 +23077,13 @@
         </is>
       </c>
       <c r="N165" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O165" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R165" t="n">
-        <v>0.0004668273620270607</v>
+        <v>0.004201446258243547</v>
       </c>
       <c r="AA165" t="inlineStr">
         <is>
@@ -23140,6 +23140,276 @@
         </is>
       </c>
       <c r="BC165" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>D052</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Chikungunya</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>基孔肯雅热</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>1079</v>
+      </c>
+      <c r="O166" t="n">
+        <v>1079</v>
+      </c>
+      <c r="R166" t="n">
+        <v>0.5037067236271986</v>
+      </c>
+      <c r="AA166" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO166" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP166" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS166" t="inlineStr"/>
+      <c r="AT166" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV166" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW166" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX166" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY166" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ166" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA166" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB166" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC166" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>1</v>
+      </c>
+      <c r="O167" t="n">
+        <v>1</v>
+      </c>
+      <c r="R167" t="n">
+        <v>0.0004668273620270607</v>
+      </c>
+      <c r="AA167" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO167" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP167" t="inlineStr">
+        <is>
+          <t>published_series</t>
+        </is>
+      </c>
+      <c r="AS167" t="inlineStr"/>
+      <c r="AT167" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY167" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ167" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA167" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB167" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC167" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -23261,7 +23531,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10">
@@ -23271,7 +23541,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11">
@@ -23323,7 +23593,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1290455</v>
+        <v>1348320</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-24 13:41:50 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -17776,13 +17776,13 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>32612</v>
+        <v>31849</v>
       </c>
       <c r="O126" t="n">
-        <v>32612</v>
+        <v>31849</v>
       </c>
       <c r="R126" t="n">
-        <v>15.22417393042651</v>
+        <v>14.86798465319986</v>
       </c>
       <c r="AA126" t="inlineStr">
         <is>
@@ -18316,13 +18316,13 @@
         </is>
       </c>
       <c r="N130" t="n">
-        <v>1100</v>
+        <v>1225</v>
       </c>
       <c r="O130" t="n">
-        <v>1100</v>
+        <v>1225</v>
       </c>
       <c r="R130" t="n">
-        <v>0.5135100982297668</v>
+        <v>0.5718635184831494</v>
       </c>
       <c r="AA130" t="inlineStr">
         <is>
@@ -18451,13 +18451,13 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>9468</v>
+        <v>9620</v>
       </c>
       <c r="O131" t="n">
-        <v>9468</v>
+        <v>9620</v>
       </c>
       <c r="R131" t="n">
-        <v>4.419921463672211</v>
+        <v>4.490879222700324</v>
       </c>
       <c r="AA131" t="inlineStr">
         <is>
@@ -20908,13 +20908,13 @@
         </is>
       </c>
       <c r="N149" t="n">
-        <v>31476</v>
+        <v>29554</v>
       </c>
       <c r="O149" t="n">
-        <v>31476</v>
+        <v>29554</v>
       </c>
       <c r="R149" t="n">
-        <v>14.69385804716376</v>
+        <v>13.79661585734775</v>
       </c>
       <c r="AA149" t="inlineStr">
         <is>
@@ -21448,13 +21448,13 @@
         </is>
       </c>
       <c r="N153" t="n">
-        <v>425</v>
+        <v>615</v>
       </c>
       <c r="O153" t="n">
-        <v>425</v>
+        <v>615</v>
       </c>
       <c r="R153" t="n">
-        <v>0.1984016288615008</v>
+        <v>0.2870988276466424</v>
       </c>
       <c r="AA153" t="inlineStr">
         <is>
@@ -21583,13 +21583,13 @@
         </is>
       </c>
       <c r="N154" t="n">
-        <v>6782</v>
+        <v>7108</v>
       </c>
       <c r="O154" t="n">
-        <v>6782</v>
+        <v>7108</v>
       </c>
       <c r="R154" t="n">
-        <v>3.166023169267526</v>
+        <v>3.318208889288348</v>
       </c>
       <c r="AA154" t="inlineStr">
         <is>
@@ -22942,13 +22942,13 @@
         </is>
       </c>
       <c r="N164" t="n">
-        <v>9847</v>
+        <v>17410</v>
       </c>
       <c r="O164" t="n">
-        <v>9847</v>
+        <v>17410</v>
       </c>
       <c r="R164" t="n">
-        <v>4.596849033880467</v>
+        <v>8.127464372891128</v>
       </c>
       <c r="AA164" t="inlineStr">
         <is>
@@ -23077,13 +23077,13 @@
         </is>
       </c>
       <c r="N165" t="n">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="O165" t="n">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="R165" t="n">
-        <v>0.004201446258243547</v>
+        <v>0.02100723129121774</v>
       </c>
       <c r="AA165" t="inlineStr">
         <is>
@@ -23212,13 +23212,13 @@
         </is>
       </c>
       <c r="N166" t="n">
-        <v>1079</v>
+        <v>2340</v>
       </c>
       <c r="O166" t="n">
-        <v>1079</v>
+        <v>2340</v>
       </c>
       <c r="R166" t="n">
-        <v>0.5037067236271986</v>
+        <v>1.092376027143322</v>
       </c>
       <c r="AA166" t="inlineStr">
         <is>
@@ -23593,7 +23593,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1348320</v>
+        <v>1355288</v>
       </c>
     </row>
     <row r="16">

</xml_diff>